<commit_message>
Update trabalho de matematica dados.xlsx
</commit_message>
<xml_diff>
--- a/trabalho de matematica dados.xlsx
+++ b/trabalho de matematica dados.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Pedro Vitor Ortiz\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C1139B2-6217-493D-8292-A2CF41A58D02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79267D49-6642-41AD-977F-CCE7346FF3E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{689BB34E-0E18-4B3F-9640-5C22EDA1B746}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>notas</t>
   </si>
@@ -63,46 +63,22 @@
     <t>F 3</t>
   </si>
   <si>
-    <t>0.985029</t>
-  </si>
-  <si>
     <t>F# 3</t>
   </si>
   <si>
-    <t>0.929744</t>
-  </si>
-  <si>
     <t>G 3</t>
   </si>
   <si>
-    <t>0.877561</t>
-  </si>
-  <si>
     <t>G# 3</t>
   </si>
   <si>
-    <t>0.828308</t>
-  </si>
-  <si>
     <t>A 3</t>
   </si>
   <si>
-    <t>0.781818</t>
-  </si>
-  <si>
     <t>A# 3</t>
   </si>
   <si>
-    <t>0.737938</t>
-  </si>
-  <si>
     <t>B 3</t>
-  </si>
-  <si>
-    <t>0.696521</t>
-  </si>
-  <si>
-    <t>comprimento de onda (m)</t>
   </si>
   <si>
     <t>344 m/s</t>
@@ -124,7 +100,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -158,6 +134,22 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -244,16 +236,18 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="3">
+  <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="2" fontId="2" fillId="2" borderId="3"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -285,9 +279,11 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="44" fontId="2" fillId="5" borderId="3" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="44" fontId="6" fillId="5" borderId="3" xfId="2" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="3">
-    <cellStyle name="Estilo 1" xfId="2" xr:uid="{4DEB79C9-2998-4324-AA2B-B2409EF3AAA8}"/>
+  <cellStyles count="4">
+    <cellStyle name="Estilo 1" xfId="3" xr:uid="{4DEB79C9-2998-4324-AA2B-B2409EF3AAA8}"/>
+    <cellStyle name="Hiperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -601,257 +597,216 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8992B49F-851A-4F89-B8AB-AAFD4B766DDD}">
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="18.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="13.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="23.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="56.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="4" max="4" width="58.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="D1" s="13" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="5">
+      <c r="B2" s="6">
         <v>277</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="6">
         <v>3.6101083032490976E-3</v>
       </c>
-      <c r="D2" s="8">
-        <v>1241059</v>
-      </c>
-      <c r="E2" s="12" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6" t="s">
+      <c r="D2" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="B3" s="7">
+      <c r="B3" s="8">
         <v>293</v>
       </c>
-      <c r="C3" s="7">
+      <c r="C3" s="8">
         <v>3.4129692832764505E-3</v>
       </c>
-      <c r="D3" s="9">
-        <v>1171404</v>
-      </c>
-      <c r="E3"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="D3"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="5">
+      <c r="B4" s="6">
         <v>311</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="6">
         <v>3.2154340836012861E-3</v>
       </c>
-      <c r="D4" s="8">
-        <v>1105658</v>
-      </c>
-      <c r="E4" s="12" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6" t="s">
+      <c r="D4" s="13" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="7">
+      <c r="B5" s="8">
         <v>329</v>
       </c>
-      <c r="C5" s="7">
+      <c r="C5" s="8">
         <v>3.0395136778115501E-3</v>
       </c>
-      <c r="D5" s="9">
-        <v>1043602</v>
-      </c>
-      <c r="E5" s="12" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
+      <c r="D5" s="14" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="5">
+      <c r="B6" s="6">
         <v>349</v>
       </c>
-      <c r="C6" s="5">
+      <c r="C6" s="6">
         <v>2.8653295128939827E-3</v>
       </c>
-      <c r="D6" s="8" t="s">
+      <c r="D6"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="E6"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6" t="s">
+      <c r="B7" s="8">
+        <v>369</v>
+      </c>
+      <c r="C7" s="8">
+        <v>2.7100271002710027E-3</v>
+      </c>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="7">
-        <v>369</v>
-      </c>
-      <c r="C7" s="7">
-        <v>2.7100271002710027E-3</v>
-      </c>
-      <c r="D7" s="9" t="s">
+      <c r="B8" s="11">
+        <v>391</v>
+      </c>
+      <c r="C8" s="6">
+        <v>2.5575447570332483E-3</v>
+      </c>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E7"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
+      <c r="B9" s="12">
+        <v>415</v>
+      </c>
+      <c r="C9" s="6">
+        <v>2.4096385542168677E-3</v>
+      </c>
+      <c r="D9"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="B8" s="10">
-        <v>391</v>
-      </c>
-      <c r="C8" s="5">
-        <v>2.5575447570332483E-3</v>
-      </c>
-      <c r="D8" s="8" t="s">
+      <c r="B10" s="11">
+        <v>440</v>
+      </c>
+      <c r="C10" s="6">
+        <v>2.2727272727272726E-3</v>
+      </c>
+      <c r="D10" s="2"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E8"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="9" t="s">
+      <c r="B11" s="12">
+        <v>466</v>
+      </c>
+      <c r="C11" s="6">
+        <v>2.1459227467811159E-3</v>
+      </c>
+      <c r="D11"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" s="11">
-        <v>415</v>
-      </c>
-      <c r="C9" s="5">
-        <v>2.4096385542168677E-3</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>14</v>
-      </c>
-      <c r="E9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="8" t="s">
-        <v>15</v>
-      </c>
-      <c r="B10" s="10">
-        <v>440</v>
-      </c>
-      <c r="C10" s="5">
-        <v>2.2727272727272726E-3</v>
-      </c>
-      <c r="D10" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="E10"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="B11" s="11">
-        <v>466</v>
-      </c>
-      <c r="C11" s="5">
-        <v>2.1459227467811159E-3</v>
-      </c>
-      <c r="D11" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="E11"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B12" s="10">
+      <c r="B12" s="11">
         <v>493</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="6">
         <v>2.0283975659229209E-3</v>
       </c>
-      <c r="D12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="D12"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A13"/>
       <c r="B13"/>
       <c r="C13"/>
       <c r="D13"/>
-      <c r="E13"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A14"/>
       <c r="B14"/>
       <c r="C14"/>
       <c r="D14"/>
-      <c r="E14"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A15"/>
       <c r="B15"/>
       <c r="C15"/>
       <c r="D15"/>
-      <c r="E15"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A16"/>
       <c r="B16"/>
       <c r="C16"/>
       <c r="D16"/>
-      <c r="E16"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17"/>
       <c r="B17"/>
       <c r="C17"/>
       <c r="D17"/>
-      <c r="E17"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18"/>
       <c r="B18"/>
       <c r="C18"/>
       <c r="D18"/>
-      <c r="E18"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19"/>
       <c r="B19"/>
       <c r="C19"/>
       <c r="D19"/>
-      <c r="E19"/>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="7" type="noConversion"/>
+  <hyperlinks>
+    <hyperlink ref="D5" r:id="rId1" xr:uid="{CACA5D8B-9DF6-4E5B-BC8D-1C82F77403EE}"/>
+  </hyperlinks>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>